<commit_message>
Auto Update Vercel Bot
</commit_message>
<xml_diff>
--- a/LINE_Bot_內容對照表.xlsx
+++ b/LINE_Bot_內容對照表.xlsx
@@ -8350,11 +8350,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A94:H94"/>
     <mergeCell ref="A106:H106"/>
     <mergeCell ref="A53:H53"/>
@@ -8362,6 +8357,11 @@
     <mergeCell ref="A73:H73"/>
     <mergeCell ref="A80:H80"/>
     <mergeCell ref="A85:H85"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A38:H38"/>
   </mergeCells>
   <phoneticPr fontId="22" type="noConversion"/>
   <hyperlinks>

</xml_diff>